<commit_message>
Bump submodule: gain normalization + clamp auto-link; K-estimator spec; sheet update
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/control_seoungjin/gain_sheet.xlsx
+++ b/control_seoungjin/gain_sheet.xlsx
@@ -644,7 +644,7 @@
       </c>
       <c r="F7" s="2" t="inlineStr">
         <is>
-          <t>플랜트 이득 음수(b=-0.0296 실측). 부호 고치면 즉시 발산 (기록 필독)</t>
+          <t>플랜트 이득 음수(b=-0.0296 실측). 부호 고치면 즉시 발산 (기록 필독) | parameters.m에선 '기본값 x sT' 식 - 기본값 숫자만 깎을 것</t>
         </is>
       </c>
     </row>
@@ -670,7 +670,7 @@
       </c>
       <c r="F8" s="4" t="inlineStr">
         <is>
-          <t>14차 채택: 활공 정상오차 소거+트림. anti-windup 없음 주의. -30은 과보상</t>
+          <t>14차 채택: 활공 정상오차 소거+트림. anti-windup 없음 주의. -30은 과보상 | parameters.m에선 '기본값 x sT' 식 - 기본값 숫자만 깎을 것</t>
         </is>
       </c>
     </row>
@@ -694,7 +694,11 @@
           <t>음수 필수!</t>
         </is>
       </c>
-      <c r="F9" s="4" t="inlineStr"/>
+      <c r="F9" s="4" t="inlineStr">
+        <is>
+          <t>parameters.m에선 '기본값 x sT' 식 - 기본값 숫자만 깎을 것</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="4" t="inlineStr">
@@ -766,7 +770,7 @@
       </c>
       <c r="F12" s="2" t="inlineStr">
         <is>
-          <t>12차 스윕 1위 (20은 수확역전)</t>
+          <t>12차 스윕 1위 (20은 수확역전) | 'x sQ' 식 - 기본값 숫자만 깎을 것</t>
         </is>
       </c>
     </row>
@@ -792,7 +796,7 @@
       </c>
       <c r="F13" s="4" t="inlineStr">
         <is>
-          <t>지속외란 필수 (PD만으론 42~65도 고착). anti-windup 없음</t>
+          <t>지속외란 필수 (PD만으론 42~65도 고착). anti-windup 없음 | 'x sQ' 식 - 기본값 숫자만 깎을 것</t>
         </is>
       </c>
     </row>
@@ -816,7 +820,11 @@
           <t>양수</t>
         </is>
       </c>
-      <c r="F14" s="4" t="inlineStr"/>
+      <c r="F14" s="4" t="inlineStr">
+        <is>
+          <t>'x sQ' 식 - 기본값 숫자만 깎을 것</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="4" t="inlineStr">
@@ -878,7 +886,11 @@
           <t>양수</t>
         </is>
       </c>
-      <c r="F17" s="2" t="inlineStr"/>
+      <c r="F17" s="2" t="inlineStr">
+        <is>
+          <t>'x sT' 식 - 기본값 숫자만 깎을 것</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="4" t="inlineStr">
@@ -900,7 +912,11 @@
           <t>양수</t>
         </is>
       </c>
-      <c r="F18" s="4" t="inlineStr"/>
+      <c r="F18" s="4" t="inlineStr">
+        <is>
+          <t>'x sT' 식 - 기본값 숫자만 깎을 것</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="4" t="inlineStr">
@@ -924,7 +940,7 @@
       </c>
       <c r="F19" s="4" t="inlineStr">
         <is>
-          <t>12차 수술: 0.3-&gt;0.15가 6.87Hz 지터 진범 잡음. 되돌리기 금물</t>
+          <t>12차 수술: 0.3-&gt;0.15가 6.87Hz 지터 진범 잡음. 되돌리기 금물 | 'x sT' 식 - 기본값 숫자만 깎을 것</t>
         </is>
       </c>
     </row>
@@ -1086,12 +1102,12 @@
       </c>
       <c r="B27" s="2" t="inlineStr">
         <is>
-          <t>PosErr Sat X/Y/Z</t>
+          <t>posErrSat (= 1.2 / kp_position)</t>
         </is>
       </c>
       <c r="C27" s="2" t="inlineStr">
         <is>
-          <t>±0.15 m</t>
+          <t>0.15 m (자동)</t>
         </is>
       </c>
       <c r="D27" s="3" t="inlineStr"/>
@@ -1102,7 +1118,7 @@
       </c>
       <c r="F27" s="2" t="inlineStr">
         <is>
-          <t>15차 Sat Z 채택. 줄이는 방향은 실험으로 기각됨(활공 악화)</t>
+          <t>15차: kp_position과 곱 불변식(C x kp = 1.2, 최대 P항 기울기 16.8도)으로 자동 연동 - 직접 수정 금지, kp만 깎으면 따라옴</t>
         </is>
       </c>
     </row>
@@ -1407,7 +1423,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A10"/>
+  <dimension ref="A1:A15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="110" customWidth="1" min="1" max="1"/>
@@ -1420,9 +1436,7 @@
         </is>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" t="inlineStr"/>
-    </row>
+    <row r="2"/>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
@@ -1465,13 +1479,42 @@
         </is>
       </c>
     </row>
-    <row r="9">
-      <c r="A9" t="inlineStr"/>
-    </row>
+    <row r="9"/>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
           <t>참고 플랜트 실측치: u-&gt;pitch 가속 이득 b = -0.0296 (11차 스텝 회귀) / 짐 모드 1.75~1.80Hz / 호버 모터 62%(635/1025 rad/s)</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr"/>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>[15차 갱신] parameters.m 구조 변화 주의:</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>- 자세/고도 게인은 '기본값 x sT', yaw는 'x sQ' 식으로 정규화됨 (K_thrust/K_drag 재추정 시 자동 보상용) - 깎을 때 식은 두고 앞의 기본값 숫자만 수정</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>- 오차 클램프는 posErrSat = 1.2/kp_position으로 자동 연동 (.slx가 변수 참조) - kp_position 깎으면 클램프가 알아서 따라옴, 직접 만지지 말 것</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>- Kthrust_ref/Kdrag_ref 앵커는 절대 갱신 금지 (튜닝 당시 기준값)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Bump submodule: attitude gain refinement adopted (38x hover jitter); sheet updated
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/control_seoungjin/gain_sheet.xlsx
+++ b/control_seoungjin/gain_sheet.xlsx
@@ -633,8 +633,10 @@
           <t>kp_attitude</t>
         </is>
       </c>
-      <c r="C7" s="2" t="n">
-        <v>-100</v>
+      <c r="C7" s="2" t="inlineStr">
+        <is>
+          <t>-85</t>
+        </is>
       </c>
       <c r="D7" s="3" t="inlineStr"/>
       <c r="E7" s="2" t="inlineStr">
@@ -644,7 +646,7 @@
       </c>
       <c r="F7" s="2" t="inlineStr">
         <is>
-          <t>플랜트 이득 음수(b=-0.0296 실측). 부호 고치면 즉시 발산 (기록 필독) | parameters.m에선 '기본값 x sT' 식 - 기본값 숫자만 깎을 것</t>
+          <t>16차 좌표하강: -100 부근 모터공진 이탈. 호버 지터 38배 개선, 절벽(-95~-90)에서 10% 여유 | 플랜트 이득 음수(b=-0.0296 실측). 부호 고치면 즉시 발산 (기록 필독) | parameters.m에선 '기본값 x sT' 식 - 기본값 숫자만 깎을 것</t>
         </is>
       </c>
     </row>
@@ -685,8 +687,10 @@
           <t>kd_attitude</t>
         </is>
       </c>
-      <c r="C9" s="4" t="n">
-        <v>-150</v>
+      <c r="C9" s="4" t="inlineStr">
+        <is>
+          <t>-127.5</t>
+        </is>
       </c>
       <c r="D9" s="3" t="inlineStr"/>
       <c r="E9" s="4" t="inlineStr">
@@ -696,7 +700,7 @@
       </c>
       <c r="F9" s="4" t="inlineStr">
         <is>
-          <t>parameters.m에선 '기본값 x sT' 식 - 기본값 숫자만 깎을 것</t>
+          <t>16차: kd/kp 비율 1.5 골짜기 바닥 | parameters.m에선 '기본값 x sT' 식 - 기본값 숫자만 깎을 것</t>
         </is>
       </c>
     </row>
@@ -711,8 +715,10 @@
           <t>filtD_attitude</t>
         </is>
       </c>
-      <c r="C10" s="4" t="n">
-        <v>2000</v>
+      <c r="C10" s="4" t="inlineStr">
+        <is>
+          <t>2500</t>
+        </is>
       </c>
       <c r="D10" s="3" t="inlineStr"/>
       <c r="E10" s="4" t="inlineStr">
@@ -722,7 +728,7 @@
       </c>
       <c r="F10" s="4" t="inlineStr">
         <is>
-          <t>12차 스윕 승자 (1000 대비 RMS 10% 개선)</t>
+          <t>16차: 1R 최선 (영향 미미) | 12차 스윕 승자 (1000 대비 RMS 10% 개선)</t>
         </is>
       </c>
     </row>
@@ -1436,7 +1442,6 @@
         </is>
       </c>
     </row>
-    <row r="2"/>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
@@ -1479,7 +1484,6 @@
         </is>
       </c>
     </row>
-    <row r="9"/>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
@@ -1487,9 +1491,7 @@
         </is>
       </c>
     </row>
-    <row r="11">
-      <c r="A11" t="inlineStr"/>
-    </row>
+    <row r="11"/>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>

</xml_diff>